<commit_message>
Cerrar evidencias y documentación final
</commit_message>
<xml_diff>
--- a/PRUEBAS.xlsx
+++ b/PRUEBAS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="PRUEBAS" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRUEBAS!$A$1:$G$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRUEBAS!$A$1:$G$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -850,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
@@ -1987,8 +1987,283 @@
         <v>148</v>
       </c>
     </row>
+    <row r="50" spans="1:7" ht="180" customHeight="1">
+      <c r="A50" s="2">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Suite automatizada consolidada en Docker</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutar ./scripts/run-tests.sh dentro de Docker linux/amd64.</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Compilaciones correctas y todas las suites aprobadas.</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>318 pruebas aprobadas: Java 43; .NET 46; cargas-python 88; transportista 49; Mongo/seed 25; web-host 40; admin-mfe 27.</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions / scripts/run-tests.sh; Compilación y pruebas Docker #3; commit c90ee33.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="180" customHeight="1">
+      <c r="A51" s="2">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>CI GitHub Actions - Compilación y pruebas Docker #3</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Workflow Compilación y pruebas Docker #3; commit c90ee33.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Compilación y pruebas Docker completadas correctamente.</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS; 318 pruebas aprobadas; commit c90ee33.</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions: Compilación y pruebas Docker #3; commit c90ee33; .github/workflows/ci.yml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="180" customHeight="1">
+      <c r="A52" s="2">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Publicación GHCR y verificación por digest - pedidos-java</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/pedidos-java:1.0.0
+Digest: sha256:1b06b858aef3638ca369b519f2aaddf87357c37453f8a6f74ce7784923466c4e
+Plataforma: linux/amd64
+Descargar por digest y arrancar con docker compose up -d --no-build --wait.</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Descarga por digest OK; arranque por digest OK; healthy OK; docker inspect coincide con el digest publicado.</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/pedidos-java:1.0.0
+Digest: sha256:1b06b858aef3638ca369b519f2aaddf87357c37453f8a6f74ce7784923466c4e
+Plataforma: linux/amd64
+Descarga por digest OK; arranque por digest OK; healthy OK. docker inspect confirmó la referencia exacta.</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions: Publicar imágenes Docker #1 SUCCESS, 5/5 jobs. Verificación real comunicada por el responsable: descarga, arranque y docker inspect de ghcr.io/informaticacinco/pedidos-java@sha256:1b06b858aef3638ca369b519f2aaddf87357c37453f8a6f74ce7784923466c4e.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="180" customHeight="1">
+      <c r="A53" s="2">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Publicación GHCR y verificación por digest - despachos-dotnet</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/despachos-dotnet:1.0.0
+Digest: sha256:88e8cfe6b6ffd6723f80211e40efd045fd506be9404235c14cbb390f9a8ac216
+Plataforma: linux/amd64
+Descargar por digest y arrancar con docker compose up -d --no-build --wait.</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Descarga por digest OK; arranque por digest OK; healthy OK; docker inspect coincide con el digest publicado.</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/despachos-dotnet:1.0.0
+Digest: sha256:88e8cfe6b6ffd6723f80211e40efd045fd506be9404235c14cbb390f9a8ac216
+Plataforma: linux/amd64
+Descarga por digest OK; arranque por digest OK; healthy OK. docker inspect confirmó la referencia exacta.</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions: Publicar imágenes Docker #1 SUCCESS, 5/5 jobs. Verificación real comunicada por el responsable: descarga, arranque y docker inspect de ghcr.io/informaticacinco/despachos-dotnet@sha256:88e8cfe6b6ffd6723f80211e40efd045fd506be9404235c14cbb390f9a8ac216.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="180" customHeight="1">
+      <c r="A54" s="2">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Publicación GHCR y verificación por digest - cargas-python</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/cargas-python:1.0.0
+Digest: sha256:8e0eae0c9fd9c736b09ea70302c8a2a4e8bed400e6e2586a0226aefd9673667b
+Plataforma: linux/amd64
+Descargar por digest y arrancar con docker compose up -d --no-build --wait.</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Descarga por digest OK; arranque por digest OK; healthy OK; docker inspect coincide con el digest publicado.</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/cargas-python:1.0.0
+Digest: sha256:8e0eae0c9fd9c736b09ea70302c8a2a4e8bed400e6e2586a0226aefd9673667b
+Plataforma: linux/amd64
+Descarga por digest OK; arranque por digest OK; healthy OK. docker inspect confirmó la referencia exacta.</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions: Publicar imágenes Docker #1 SUCCESS, 5/5 jobs. Verificación real comunicada por el responsable: descarga, arranque y docker inspect de ghcr.io/informaticacinco/cargas-python@sha256:8e0eae0c9fd9c736b09ea70302c8a2a4e8bed400e6e2586a0226aefd9673667b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="180" customHeight="1">
+      <c r="A55" s="2">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Publicación GHCR y verificación por digest - web-host</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/web-host:1.0.0
+Digest: sha256:3a21700d69821a896bea495c81541e290d3a278f6199854d4e76d38e25a609f6
+Plataforma: linux/amd64
+Descargar por digest y arrancar con docker compose up -d --no-build --wait.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Descarga por digest OK; arranque por digest OK; healthy OK; docker inspect coincide con el digest publicado.</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/web-host:1.0.0
+Digest: sha256:3a21700d69821a896bea495c81541e290d3a278f6199854d4e76d38e25a609f6
+Plataforma: linux/amd64
+Descarga por digest OK; arranque por digest OK; healthy OK. docker inspect confirmó la referencia exacta.</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions: Publicar imágenes Docker #1 SUCCESS, 5/5 jobs. Verificación real comunicada por el responsable: descarga, arranque y docker inspect de ghcr.io/informaticacinco/web-host@sha256:3a21700d69821a896bea495c81541e290d3a278f6199854d4e76d38e25a609f6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="180" customHeight="1">
+      <c r="A56" s="2">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Publicación GHCR y verificación por digest - admin-mfe</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/admin-mfe:1.0.0
+Digest: sha256:eccd27db108fdef49bff498a44540c77af920ce5da2d95826a0e2b90d6ee51a9
+Plataforma: linux/amd64
+Descargar por digest y arrancar con docker compose up -d --no-build --wait.</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Descarga por digest OK; arranque por digest OK; healthy OK; docker inspect coincide con el digest publicado.</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Imagen: ghcr.io/informaticacinco/admin-mfe:1.0.0
+Digest: sha256:eccd27db108fdef49bff498a44540c77af920ce5da2d95826a0e2b90d6ee51a9
+Plataforma: linux/amd64
+Descarga por digest OK; arranque por digest OK; healthy OK. docker inspect confirmó la referencia exacta.</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions: Publicar imágenes Docker #1 SUCCESS, 5/5 jobs. Verificación real comunicada por el responsable: descarga, arranque y docker inspect de ghcr.io/informaticacinco/admin-mfe@sha256:eccd27db108fdef49bff498a44540c77af920ce5da2d95826a0e2b90d6ee51a9.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G49"/>
+  <autoFilter ref="A1:G56"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>